<commit_message>
Standardized raw data's columns. Added a description for Data Wrangling.
</commit_message>
<xml_diff>
--- a/data/raw/task_1_raw.xlsx
+++ b/data/raw/task_1_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eckspur\Documents\!UNIVERSITY\HIT140 (Foundations of Data Science)\ASSIGNMENT 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eckspur\Documents\!UNIVERSITY\HIT140 (Foundations of Data Science)\FIFA-2026-PROJECT\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B0E469-F1A8-43FB-A755-94595CF90B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD96034F-83C7-448C-8ED8-8988F00EB91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,12 +25,6 @@
     <t>TEAMS</t>
   </si>
   <si>
-    <t>GROUP STAGE MATCHES</t>
-  </si>
-  <si>
-    <t>GROUP STAGE GOALS</t>
-  </si>
-  <si>
     <t>QUALIFIED</t>
   </si>
   <si>
@@ -182,6 +176,12 @@
   </si>
   <si>
     <t>Panama</t>
+  </si>
+  <si>
+    <t>GROUP_STAGE_MATCHES</t>
+  </si>
+  <si>
+    <t>GROUP_STAGE_GOALS</t>
   </si>
 </sst>
 </file>
@@ -569,18 +569,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" s="3">
         <v>3</v>
@@ -589,12 +589,12 @@
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" s="3">
         <v>3</v>
@@ -603,12 +603,12 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
@@ -617,12 +617,12 @@
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3">
         <v>3</v>
@@ -631,12 +631,12 @@
         <v>2</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3">
         <v>3</v>
@@ -645,12 +645,12 @@
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3">
         <v>3</v>
@@ -659,12 +659,12 @@
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3">
         <v>3</v>
@@ -673,12 +673,12 @@
         <v>5</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3">
         <v>3</v>
@@ -687,12 +687,12 @@
         <v>2</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10" s="3">
         <v>3</v>
@@ -701,12 +701,12 @@
         <v>7</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11" s="3">
         <v>3</v>
@@ -715,12 +715,12 @@
         <v>6</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" s="3">
         <v>3</v>
@@ -729,12 +729,12 @@
         <v>1</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13" s="3">
         <v>3</v>
@@ -743,12 +743,12 @@
         <v>2</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B14" s="3">
         <v>3</v>
@@ -757,12 +757,12 @@
         <v>8</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15" s="3">
         <v>3</v>
@@ -771,12 +771,12 @@
         <v>2</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16" s="3">
         <v>3</v>
@@ -785,12 +785,12 @@
         <v>2</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
@@ -799,12 +799,12 @@
         <v>3</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
@@ -813,12 +813,12 @@
         <v>11</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19" s="3">
         <v>3</v>
@@ -827,12 +827,12 @@
         <v>4</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" s="3">
         <v>3</v>
@@ -841,12 +841,12 @@
         <v>2</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" s="3">
         <v>3</v>
@@ -855,12 +855,12 @@
         <v>1</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B22" s="3">
         <v>3</v>
@@ -869,12 +869,12 @@
         <v>10</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B23" s="3">
         <v>3</v>
@@ -883,12 +883,12 @@
         <v>7</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B24" s="3">
         <v>3</v>
@@ -897,12 +897,12 @@
         <v>7</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B25" s="3">
         <v>3</v>
@@ -911,12 +911,12 @@
         <v>2</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B26" s="3">
         <v>3</v>
@@ -925,12 +925,12 @@
         <v>6</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B27" s="3">
         <v>3</v>
@@ -939,12 +939,12 @@
         <v>5</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B28" s="3">
         <v>3</v>
@@ -953,12 +953,12 @@
         <v>3</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B29" s="3">
         <v>3</v>
@@ -967,12 +967,12 @@
         <v>4</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B30" s="3">
         <v>3</v>
@@ -981,12 +981,12 @@
         <v>5</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B31" s="3">
         <v>3</v>
@@ -995,12 +995,12 @@
         <v>4</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B32" s="3">
         <v>3</v>
@@ -1009,12 +1009,12 @@
         <v>3</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B33" s="3">
         <v>3</v>
@@ -1023,12 +1023,12 @@
         <v>1</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B34" s="3">
         <v>3</v>
@@ -1037,12 +1037,12 @@
         <v>10</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B35" s="3">
         <v>3</v>
@@ -1051,12 +1051,12 @@
         <v>8</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B36" s="3">
         <v>3</v>
@@ -1065,12 +1065,12 @@
         <v>8</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B37" s="3">
         <v>3</v>
@@ -1079,12 +1079,12 @@
         <v>1</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B38" s="3">
         <v>3</v>
@@ -1093,12 +1093,12 @@
         <v>8</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B39" s="3">
         <v>3</v>
@@ -1107,12 +1107,12 @@
         <v>6</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B40" s="3">
         <v>3</v>
@@ -1121,12 +1121,12 @@
         <v>5</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B41" s="3">
         <v>3</v>
@@ -1135,12 +1135,12 @@
         <v>3</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B42" s="3">
         <v>3</v>
@@ -1149,12 +1149,12 @@
         <v>6</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B43" s="3">
         <v>3</v>
@@ -1163,12 +1163,12 @@
         <v>6</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B44" s="3">
         <v>3</v>
@@ -1177,12 +1177,12 @@
         <v>4</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B45" s="3">
         <v>3</v>
@@ -1191,12 +1191,12 @@
         <v>2</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B46" s="3">
         <v>3</v>
@@ -1205,12 +1205,12 @@
         <v>6</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B47" s="3">
         <v>3</v>
@@ -1219,12 +1219,12 @@
         <v>5</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B48" s="3">
         <v>3</v>
@@ -1233,12 +1233,12 @@
         <v>2</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B49" s="3">
         <v>3</v>
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>